<commit_message>
feat: release v0.2.0 with CaveAgent, SABER, ReCode DAG (Score: 73.7)
</commit_message>
<xml_diff>
--- a/internal/sheet/testdata/simple.xlsx
+++ b/internal/sheet/testdata/simple.xlsx
@@ -1,15 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="true" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10215"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2DD6F74-DC4C-D445-81F8-A597CDDF8963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="14800" windowHeight="8020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="122211"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -34,13 +48,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="FangSong"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="2">
@@ -67,15 +87,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -331,11 +359,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -346,7 +374,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -357,7 +385,7 @@
         <v>90.5</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -368,11 +396,14 @@
         <v>85</v>
       </c>
     </row>
-    <row r="4">
-      <c r="C4" t="str">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C4">
         <f>SUM(C2:C3)</f>
+        <v>175.5</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>